<commit_message>
feat(F-NAR-009): SAN.ECR.001-06–10 et HYG.001-01/02
Ouvertures monde d’abord (livre en tissu, soupe, couverture, lampe,
pain, carreaux, gravier). Audio plus tard.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-SAN.ECR.001-06.xlsx
+++ b/stories/arbres/ATOM-SAN.ECR.001-06.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Anouk éteint et prend un livre</t>
+          <t>Le livre en tissu</t>
         </is>
       </c>
     </row>
@@ -830,6 +830,18 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>voix-roles-v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fil_rouge</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Un livre en tissu attend. Maman dit fini. Nina éteint. Elle tourne une page. Le lapin est là.</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1184,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Anouk est dans le coin lecture. Elle regarde un dessin sur la tablette. Un oiseau chante dans l'histoire. Le coussin est doux. Maman s'assoit près d'elle. Fini. L'adulte dit fini. Anouk écoute. Elle va éteindre. Anouk éteint l'écran. L'écran devient noir. Elle pose la tablette sur le coussin. On prend un autre jeu. Anouk choisit un livre en tissu. Le livre sent le coton. Anouk tourne une page. Maman nomme le lapin. L'écran est éteint. Un autre jeu, c'est bien. L'adulte a dit fini. Elle a éteint. Puis elle a un autre jeu. Maman tape doucement dans ses mains. Anouk rit. Le coin lecture est calme.</t>
+          <t>Un livre en tissu attend. Il est sur le gros coussin. Le coussin est tout doux. Un fil rouge dépasse un peu. La lumière passe dans le rideau. Elle est jaune et tiède. Ça sent le coton. Un oiseau tape à la vitre. Toc, toc. Le coin lecture est calme. Une chaussette rose traîne. Nina, viens. Tu vois le livre ? Oui, maman. Il est doux. En ce moment, Nina tient la tablette. Un oiseau chante dans l'histoire. Le coussin est chaud. Il chante, maman. Oui. Il chante. Maman s'assoit près d'elle. Sa robe sent le savon. Fini. L'adulte dit fini. Nina écoute. C'est fini. On va éteindre. Nina va éteindre. Nina éteint l'écran. L'écran devient noir. Elle pose la tablette. La tablette est sur le coussin. Bravo, Nina. Tu as éteint. On prend un autre jeu. Un autre jeu. Tu choisis ? Nina prend le livre en tissu. Le livre sent le coton. La page est douce. Un lapin gris est cousu. Le lapin. Oui. C'est le lapin. Il a de grandes oreilles. Nina tourne une page. Ça fait un petit bruit. Une carotte orange apparaît. Une carotte. Oui. La carotte du lapin. Bravo. Tu as fait du bon travail. L'écran est éteint. Oui. Un autre jeu, c'est bien. Maman tape doucement. Nina rit. Le coin lecture est calme. Le livre reste ouvert.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1312,13 +1324,67 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Anouk est dans le coin lecture. Elle regarde un dessin sur la tablette. Un oiseau chante dans l'histoire. Le coussin est doux. Maman s'assoit près d'elle.
-maman|Fini. L'adulte dit fini.
-narrateur|Anouk écoute. Elle va éteindre. Anouk éteint l'écran. L'écran devient noir. Elle pose la tablette sur le coussin.
+          <t>narrateur|Un livre en tissu attend.
+narrateur|Il est sur le gros coussin.
+narrateur|Le coussin est tout doux.
+narrateur|Un fil rouge dépasse un peu.
+narrateur|La lumière passe dans le rideau.
+narrateur|Elle est jaune et tiède.
+narrateur|Ça sent le coton.
+narrateur|Un oiseau tape à la vitre.
+narrateur|Toc, toc.
+narrateur|Le coin lecture est calme.
+narrateur|Une chaussette rose traîne.
+maman|Nina, viens.
+maman|Tu vois le livre ?
+enfant-f|Oui, maman.
+enfant-f|Il est doux.
+narrateur|En ce moment, Nina tient la tablette.
+narrateur|Un oiseau chante dans l'histoire.
+narrateur|Le coussin est chaud.
+enfant-f|Il chante, maman.
+maman|Oui.
+maman|Il chante.
+narrateur|Maman s'assoit près d'elle.
+narrateur|Sa robe sent le savon.
+maman|Fini.
+narrateur|L'adulte dit fini.
+narrateur|Nina écoute.
+enfant-f|C'est fini.
+maman|On va éteindre.
+narrateur|Nina va éteindre.
+narrateur|Nina éteint l'écran.
+narrateur|L'écran devient noir.
+narrateur|Elle pose la tablette.
+narrateur|La tablette est sur le coussin.
+maman|Bravo, Nina.
+maman|Tu as éteint.
 maman|On prend un autre jeu.
-narrateur|Anouk choisit un livre en tissu. Le livre sent le coton. Anouk tourne une page. Maman nomme le lapin.
-enfant-m|L'écran est éteint.
-narrateur|Un autre jeu, c'est bien. L'adulte a dit fini. Elle a éteint. Puis elle a un autre jeu. Maman tape doucement dans ses mains. Anouk rit. Le coin lecture est calme.</t>
+enfant-f|Un autre jeu.
+maman|Tu choisis ?
+narrateur|Nina prend le livre en tissu.
+narrateur|Le livre sent le coton.
+narrateur|La page est douce.
+narrateur|Un lapin gris est cousu.
+enfant-f|Le lapin.
+maman|Oui.
+maman|C'est le lapin.
+maman|Il a de grandes oreilles.
+narrateur|Nina tourne une page.
+narrateur|Ça fait un petit bruit.
+narrateur|Une carotte orange apparaît.
+enfant-f|Une carotte.
+maman|Oui.
+maman|La carotte du lapin.
+maman|Bravo.
+maman|Tu as fait du bon travail.
+enfant-f|L'écran est éteint.
+maman|Oui.
+maman|Un autre jeu, c'est bien.
+narrateur|Maman tape doucement.
+narrateur|Nina rit.
+narrateur|Le coin lecture est calme.
+narrateur|Le livre reste ouvert.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr"/>
@@ -1346,7 +1412,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Maman dit fini. Que fait Anouk ?</t>
+          <t>Maman dit fini. Que fait Nina ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1502,7 +1568,8 @@
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Maman dit fini. Que fait Anouk ?</t>
+          <t>narrateur|Maman dit fini.
+narrateur|Que fait Nina ?</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr"/>
@@ -1530,7 +1597,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Maman a dit fini. Anouk a éteint. Elle a pris un autre jeu. Le livre, c'était bien.</t>
+          <t>Maman a dit fini. L'adulte a dit fini. Nina a éteint. Elle a pris un autre jeu. Tu as éteint ? Oui, maman. Et après ? Un autre jeu. Bravo. Le livre, c'était bien. Nina touche le lapin. Le tissu est doux. Tu tournes encore une page ? Oui. La carotte est encore là. Le fil rouge brille un peu.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1674,7 +1741,22 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Maman a dit fini. Anouk a éteint. Elle a pris un autre jeu. Le livre, c'était bien.</t>
+          <t>narrateur|Maman a dit fini.
+narrateur|L'adulte a dit fini.
+narrateur|Nina a éteint.
+narrateur|Elle a pris un autre jeu.
+maman|Tu as éteint ?
+enfant-f|Oui, maman.
+maman|Et après ?
+enfant-f|Un autre jeu.
+maman|Bravo.
+maman|Le livre, c'était bien.
+narrateur|Nina touche le lapin.
+narrateur|Le tissu est doux.
+maman|Tu tournes encore une page ?
+enfant-f|Oui.
+narrateur|La carotte est encore là.
+narrateur|Le fil rouge brille un peu.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr"/>
@@ -1702,7 +1784,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Le lapin est sur la page. Anouk dit merci à maman.</t>
+          <t>Le lapin est sur la page. On range la tablette ? Nina pose la tablette. Elle la met près du rideau. Tu as fini de ranger ? Oui, maman. Bravo. Merci, maman. Merci, Nina. On referme le livre ? Nina referme le livre. Le coussin reste chaud. Ça sent encore le coton.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1838,7 +1920,19 @@
       <c r="AV5" s="2" t="inlineStr"/>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Le lapin est sur la page. Anouk dit merci à maman.</t>
+          <t>narrateur|Le lapin est sur la page.
+maman|On range la tablette ?
+narrateur|Nina pose la tablette.
+narrateur|Elle la met près du rideau.
+maman|Tu as fini de ranger ?
+enfant-f|Oui, maman.
+maman|Bravo.
+enfant-f|Merci, maman.
+maman|Merci, Nina.
+maman|On referme le livre ?
+narrateur|Nina referme le livre.
+narrateur|Le coussin reste chaud.
+narrateur|Ça sent encore le coton.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr"/>
@@ -1866,7 +1960,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>Le livre reste ouvert. Le lapin est là. Oui. Bravo, Nina. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2006,7 +2100,11 @@
       <c r="AV6" s="2" t="inlineStr"/>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
+          <t>narrateur|Le livre reste ouvert.
+enfant-f|Le lapin est là.
+maman|Oui.
+maman|Bravo, Nina.
+narrateur|L'histoire est finie.</t>
         </is>
       </c>
       <c r="AX6" t="inlineStr"/>
@@ -2028,7 +2126,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2066,6 +2164,13 @@
       <c r="A5" t="inlineStr">
         <is>
           <t>F-AUD-007 colonne sons ; vide = silence ; jamais parler dans le bruit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
         </is>
       </c>
     </row>

</xml_diff>